<commit_message>
feat(demo): a Row validation toggle with three dirty rows to catch
The sample file grows three rows a validator should flag — a duplicate id, a
missing name, a broken email — appended at the end so the preview and the
README screenshot are untouched.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/public/sample-contacts.xlsx
+++ b/demo/public/sample-contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N24"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1339,9 +1339,141 @@
         <v>44 Hawthorne St</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1020304050</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Odette</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Marchetti</v>
+      </c>
+      <c r="D22" t="str">
+        <v>REF-4220</v>
+      </c>
+      <c r="E22" t="str">
+        <v>odette.m@harborpoint.com</v>
+      </c>
+      <c r="F22" t="str">
+        <v>+1 415 555 0101</v>
+      </c>
+      <c r="G22" t="str">
+        <v>LG1040</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I22" t="str">
+        <v>1992-03-18</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Analyst</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Harbor</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Portland</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Oregon</v>
+      </c>
+      <c r="N22" t="str">
+        <v>12 Alder Ct</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1020304071</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>Nakamura</v>
+      </c>
+      <c r="D23" t="str">
+        <v>REF-4221</v>
+      </c>
+      <c r="E23" t="str">
+        <v>ken.nakamura@northgate.io</v>
+      </c>
+      <c r="F23" t="str">
+        <v>+1 206 555 0102</v>
+      </c>
+      <c r="G23" t="str">
+        <v>LG1047</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I23" t="str">
+        <v>1986-08-22</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Engineer</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Northgate</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Washington</v>
+      </c>
+      <c r="N23" t="str">
+        <v>88 Cedar Way</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1020304072</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Farida</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Benali</v>
+      </c>
+      <c r="D24" t="str">
+        <v>REF-4222</v>
+      </c>
+      <c r="E24" t="str">
+        <v>farida.benali(at)brightlane</v>
+      </c>
+      <c r="F24" t="str">
+        <v>+1 312 555 0103</v>
+      </c>
+      <c r="G24" t="str">
+        <v>LG1054</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I24" t="str">
+        <v>1995-05-09</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Coordinator</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Brightlane</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Illinois</v>
+      </c>
+      <c r="N24" t="str">
+        <v>5 Birch Row</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>